<commit_message>
lsaeb intv and stop dist can be extracted
</commit_message>
<xml_diff>
--- a/config/kpi_as_long.xlsx
+++ b/config/kpi_as_long.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wangjianhai/02_ADAS/01_repo/01_Tools/01_kpi_extractor/python/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CE815F8-B665-094E-BD5E-A8B4E80EE564}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE6BE749-7152-6444-8DAA-04D4CBC8794E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="700" windowWidth="34200" windowHeight="20360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="8700" windowWidth="34200" windowHeight="20360" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="params" sheetId="7" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="257">
   <si>
     <t>Reference</t>
   </si>
@@ -787,6 +787,33 @@
   </si>
   <si>
     <t>FB_JERK_NEG_THD</t>
+  </si>
+  <si>
+    <t>LSAEB</t>
+  </si>
+  <si>
+    <t>lsaebIntvLongDist</t>
+  </si>
+  <si>
+    <t>lsaebIntvLatDist</t>
+  </si>
+  <si>
+    <t>lsaebStopLongDist</t>
+  </si>
+  <si>
+    <t>lsaebStopLatDist</t>
+  </si>
+  <si>
+    <t>Longitudinal distance at LSAEB intervention start</t>
+  </si>
+  <si>
+    <t>Lateral distance at LSAEB intervention start</t>
+  </si>
+  <si>
+    <t>Longitudinal gap when vehicle stopped</t>
+  </si>
+  <si>
+    <t>Lateral gap when vehicle stopped</t>
   </si>
 </sst>
 </file>
@@ -2436,7 +2463,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CE39B99-0AFB-8547-83BF-D855CC6E3BB3}">
-  <dimension ref="B1:G44"/>
+  <dimension ref="B1:G48"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.83203125" style="13" customWidth="1"/>
@@ -3232,6 +3259,74 @@
       </c>
       <c r="G44" s="13" t="s">
         <v>244</v>
+      </c>
+    </row>
+    <row r="45" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B45" s="13" t="s">
+        <v>248</v>
+      </c>
+      <c r="C45" s="13" t="s">
+        <v>249</v>
+      </c>
+      <c r="D45" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="E45" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="G45" s="13" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="46" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B46" s="13" t="s">
+        <v>248</v>
+      </c>
+      <c r="C46" s="13" t="s">
+        <v>250</v>
+      </c>
+      <c r="D46" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="E46" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="G46" s="13" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="47" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B47" s="13" t="s">
+        <v>248</v>
+      </c>
+      <c r="C47" s="13" t="s">
+        <v>251</v>
+      </c>
+      <c r="D47" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="E47" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="G47" s="13" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="48" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B48" s="13" t="s">
+        <v>248</v>
+      </c>
+      <c r="C48" s="13" t="s">
+        <v>252</v>
+      </c>
+      <c r="D48" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="E48" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="G48" s="13" t="s">
+        <v>256</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
lsaeb feature integration done
</commit_message>
<xml_diff>
--- a/config/kpi_as_long.xlsx
+++ b/config/kpi_as_long.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wangjianhai/02_ADAS/01_repo/01_Tools/01_kpi_extractor/python/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE6BE749-7152-6444-8DAA-04D4CBC8794E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43707EA3-C977-F84C-A9B5-733C1DA7EC34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="8700" windowWidth="34200" windowHeight="20360" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="820" windowWidth="34200" windowHeight="20360" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="params" sheetId="7" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="540" uniqueCount="263">
   <si>
     <t>Reference</t>
   </si>
@@ -814,6 +814,24 @@
   </si>
   <si>
     <t>Lateral gap when vehicle stopped</t>
+  </si>
+  <si>
+    <t>LongInterventionDistance</t>
+  </si>
+  <si>
+    <t>LatInterventionDistance</t>
+  </si>
+  <si>
+    <t>LongStopDistance</t>
+  </si>
+  <si>
+    <t>LatStopDistance</t>
+  </si>
+  <si>
+    <t>LSAEB Long Braking Distances</t>
+  </si>
+  <si>
+    <t>LSAEB Lat Braking Distances</t>
   </si>
 </sst>
 </file>
@@ -866,7 +884,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -887,17 +905,6 @@
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -922,7 +929,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -938,7 +944,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1722,7 +1729,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24310F59-1486-4F41-B3B7-AB25CE8F592D}">
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="33.6640625" customWidth="1"/>
@@ -1785,10 +1792,10 @@
         <v>15</v>
       </c>
       <c r="D2" s="2">
-        <v>5</v>
+        <v>-10</v>
       </c>
       <c r="E2" s="2">
-        <v>85</v>
+        <v>10</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>31</v>
@@ -2419,42 +2426,208 @@
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A19" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="B19" s="9" t="s">
+      <c r="A19" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="C19" s="15" t="s">
+      <c r="C19" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="D19" s="15">
-        <v>0</v>
-      </c>
-      <c r="E19" s="15">
+      <c r="D19" s="2">
+        <v>0</v>
+      </c>
+      <c r="E19" s="2">
         <v>0.3</v>
       </c>
-      <c r="F19" s="9" t="s">
+      <c r="F19" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="G19" s="15" t="b">
+      <c r="G19" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="H19" s="9" t="s">
+      <c r="H19" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I19" s="9" t="s">
+      <c r="I19" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="J19" s="9" t="s">
+      <c r="J19" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="K19" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="L19" s="9" t="b">
-        <v>0</v>
-      </c>
+      <c r="K19" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L19" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A20" s="14" t="s">
+        <v>248</v>
+      </c>
+      <c r="B20" s="14" t="s">
+        <v>261</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="D20" s="15">
+        <v>-10</v>
+      </c>
+      <c r="E20" s="15">
+        <v>10</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G20" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I20" s="14" t="s">
+        <v>257</v>
+      </c>
+      <c r="J20" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K20" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L20" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A21" s="14" t="s">
+        <v>248</v>
+      </c>
+      <c r="B21" s="14" t="s">
+        <v>262</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="D21" s="15">
+        <v>-10</v>
+      </c>
+      <c r="E21" s="15">
+        <v>10</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G21" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I21" s="14" t="s">
+        <v>258</v>
+      </c>
+      <c r="J21" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K21" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L21" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A22" s="14" t="s">
+        <v>248</v>
+      </c>
+      <c r="B22" s="14" t="s">
+        <v>261</v>
+      </c>
+      <c r="C22" s="15" t="s">
+        <v>251</v>
+      </c>
+      <c r="D22" s="15">
+        <v>-10</v>
+      </c>
+      <c r="E22" s="15">
+        <v>10</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G22" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I22" s="14" t="s">
+        <v>259</v>
+      </c>
+      <c r="J22" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K22" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L22" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A23" s="14" t="s">
+        <v>248</v>
+      </c>
+      <c r="B23" s="14" t="s">
+        <v>262</v>
+      </c>
+      <c r="C23" s="15" t="s">
+        <v>252</v>
+      </c>
+      <c r="D23" s="15">
+        <v>-10</v>
+      </c>
+      <c r="E23" s="15">
+        <v>10</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G23" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I23" s="14" t="s">
+        <v>260</v>
+      </c>
+      <c r="J23" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K23" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L23" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A24" s="1"/>
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
+      <c r="F24" s="1"/>
+      <c r="G24" s="1"/>
+      <c r="H24" s="1"/>
+      <c r="I24" s="1"/>
+      <c r="J24" s="1"/>
+      <c r="K24" s="1"/>
+      <c r="L24" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2466,866 +2639,866 @@
   <dimension ref="B1:G48"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="2.83203125" style="13" customWidth="1"/>
-    <col min="2" max="2" width="12.1640625" style="13" customWidth="1"/>
-    <col min="3" max="3" width="17" style="13" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.5" style="13" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.1640625" style="13" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21" style="13" customWidth="1"/>
-    <col min="7" max="7" width="45.1640625" style="13" customWidth="1"/>
-    <col min="8" max="16384" width="10.83203125" style="13"/>
+    <col min="1" max="1" width="2.83203125" style="12" customWidth="1"/>
+    <col min="2" max="2" width="12.1640625" style="12" customWidth="1"/>
+    <col min="3" max="3" width="17" style="12" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.5" style="12" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.1640625" style="12" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21" style="12" customWidth="1"/>
+    <col min="7" max="7" width="45.1640625" style="12" customWidth="1"/>
+    <col min="8" max="16384" width="10.83203125" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:7" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="10" t="s">
+    <row r="1" spans="2:7" s="10" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B1" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="F1" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="G1" s="10" t="s">
+      <c r="G1" s="9" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="2" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="11" t="s">
         <v>186</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="11" t="s">
         <v>187</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="11" t="s">
         <v>188</v>
       </c>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12" t="s">
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
+      <c r="G2" s="11" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="3" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="11" t="s">
         <v>186</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="C3" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="D3" s="12" t="s">
+      <c r="D3" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="E3" s="12" t="s">
+      <c r="E3" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12" t="s">
+      <c r="F3" s="11"/>
+      <c r="G3" s="11" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="11" t="s">
         <v>186</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="D4" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="E4" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="F4" s="12"/>
-      <c r="G4" s="12" t="s">
+      <c r="F4" s="11"/>
+      <c r="G4" s="11" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B5" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C5" s="12" t="s">
+      <c r="B5" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C5" s="11" t="s">
         <v>134</v>
       </c>
-      <c r="D5" s="12" t="s">
+      <c r="D5" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="E5" s="12" t="s">
+      <c r="E5" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12" t="s">
+      <c r="F5" s="11"/>
+      <c r="G5" s="11" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B6" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C6" s="12" t="s">
+      <c r="B6" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C6" s="11" t="s">
         <v>135</v>
       </c>
-      <c r="D6" s="12" t="s">
+      <c r="D6" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="E6" s="12" t="s">
+      <c r="E6" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="F6" s="12"/>
-      <c r="G6" s="12" t="s">
+      <c r="F6" s="11"/>
+      <c r="G6" s="11" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B7" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C7" s="12" t="s">
+      <c r="B7" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C7" s="11" t="s">
         <v>136</v>
       </c>
-      <c r="D7" s="12" t="s">
+      <c r="D7" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="E7" s="12" t="s">
+      <c r="E7" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="F7" s="12"/>
-      <c r="G7" s="12" t="s">
+      <c r="F7" s="11"/>
+      <c r="G7" s="11" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B8" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C8" s="12" t="s">
+      <c r="B8" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C8" s="11" t="s">
         <v>137</v>
       </c>
-      <c r="D8" s="12" t="s">
+      <c r="D8" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="E8" s="12" t="s">
+      <c r="E8" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12" t="s">
+      <c r="F8" s="11"/>
+      <c r="G8" s="11" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B9" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C9" s="12" t="s">
+      <c r="B9" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="D9" s="12" t="s">
+      <c r="D9" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="E9" s="12" t="s">
+      <c r="E9" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="F9" s="12"/>
-      <c r="G9" s="12" t="s">
+      <c r="F9" s="11"/>
+      <c r="G9" s="11" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B10" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C10" s="12" t="s">
+      <c r="B10" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="D10" s="12" t="s">
+      <c r="D10" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="E10" s="12"/>
-      <c r="F10" s="12"/>
-      <c r="G10" s="12" t="s">
+      <c r="E10" s="11"/>
+      <c r="F10" s="11"/>
+      <c r="G10" s="11" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B11" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C11" s="12" t="s">
+      <c r="B11" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C11" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="D11" s="12" t="s">
+      <c r="D11" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12"/>
-      <c r="G11" s="12" t="s">
+      <c r="E11" s="11"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B12" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C12" s="12" t="s">
+      <c r="B12" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C12" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="D12" s="12" t="s">
+      <c r="D12" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="E12" s="12"/>
-      <c r="F12" s="12"/>
-      <c r="G12" s="12" t="s">
+      <c r="E12" s="11"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="11" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B13" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C13" s="12" t="s">
+      <c r="B13" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C13" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="D13" s="12" t="s">
+      <c r="D13" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="E13" s="12" t="s">
+      <c r="E13" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="F13" s="12"/>
-      <c r="G13" s="12" t="s">
+      <c r="F13" s="11"/>
+      <c r="G13" s="11" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B14" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C14" s="12" t="s">
+      <c r="B14" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C14" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="D14" s="12" t="s">
+      <c r="D14" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="E14" s="12" t="s">
+      <c r="E14" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="F14" s="12"/>
-      <c r="G14" s="12" t="s">
+      <c r="F14" s="11"/>
+      <c r="G14" s="11" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B15" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C15" s="12" t="s">
+      <c r="B15" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C15" s="11" t="s">
         <v>138</v>
       </c>
-      <c r="D15" s="12" t="s">
+      <c r="D15" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="E15" s="12" t="s">
+      <c r="E15" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="F15" s="12"/>
-      <c r="G15" s="12" t="s">
+      <c r="F15" s="11"/>
+      <c r="G15" s="11" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B16" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C16" s="12" t="s">
+      <c r="B16" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C16" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="D16" s="12" t="s">
+      <c r="D16" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="E16" s="12"/>
-      <c r="F16" s="12"/>
-      <c r="G16" s="12" t="s">
+      <c r="E16" s="11"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="11" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B17" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C17" s="12" t="s">
+      <c r="B17" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C17" s="11" t="s">
         <v>139</v>
       </c>
-      <c r="D17" s="12" t="s">
+      <c r="D17" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="E17" s="12" t="s">
+      <c r="E17" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="F17" s="12"/>
-      <c r="G17" s="12" t="s">
+      <c r="F17" s="11"/>
+      <c r="G17" s="11" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B18" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C18" s="12" t="s">
+      <c r="B18" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C18" s="11" t="s">
         <v>140</v>
       </c>
-      <c r="D18" s="12" t="s">
+      <c r="D18" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="E18" s="12" t="s">
+      <c r="E18" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="F18" s="12"/>
-      <c r="G18" s="12" t="s">
+      <c r="F18" s="11"/>
+      <c r="G18" s="11" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B19" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C19" s="12" t="s">
+      <c r="B19" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C19" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="D19" s="12" t="s">
+      <c r="D19" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="E19" s="12" t="s">
+      <c r="E19" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="F19" s="12" t="s">
+      <c r="F19" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="G19" s="12" t="s">
+      <c r="G19" s="11" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B20" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C20" s="12" t="s">
+      <c r="B20" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C20" s="11" t="s">
         <v>141</v>
       </c>
-      <c r="D20" s="12" t="s">
+      <c r="D20" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="E20" s="12"/>
-      <c r="F20" s="12"/>
-      <c r="G20" s="12" t="s">
+      <c r="E20" s="11"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="11" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B21" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C21" s="12" t="s">
+      <c r="B21" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C21" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="D21" s="12" t="s">
+      <c r="D21" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="E21" s="12" t="s">
+      <c r="E21" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="F21" s="12"/>
-      <c r="G21" s="12" t="s">
+      <c r="F21" s="11"/>
+      <c r="G21" s="11" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B22" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C22" s="12" t="s">
+      <c r="B22" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C22" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="D22" s="12" t="s">
+      <c r="D22" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="E22" s="12" t="s">
+      <c r="E22" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="F22" s="12" t="s">
+      <c r="F22" s="11" t="s">
         <v>131</v>
       </c>
-      <c r="G22" s="12" t="s">
+      <c r="G22" s="11" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B23" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C23" s="12" t="s">
+      <c r="B23" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C23" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="D23" s="12" t="s">
+      <c r="D23" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="E23" s="12"/>
-      <c r="F23" s="12"/>
-      <c r="G23" s="12" t="s">
+      <c r="E23" s="11"/>
+      <c r="F23" s="11"/>
+      <c r="G23" s="11" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="24" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B24" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C24" s="12" t="s">
+      <c r="B24" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C24" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="D24" s="12" t="s">
+      <c r="D24" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="E24" s="12" t="s">
+      <c r="E24" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="F24" s="12"/>
-      <c r="G24" s="12" t="s">
+      <c r="F24" s="11"/>
+      <c r="G24" s="11" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="25" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B25" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C25" s="12" t="s">
+      <c r="B25" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C25" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="D25" s="12" t="s">
+      <c r="D25" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="E25" s="12" t="s">
+      <c r="E25" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="F25" s="12" t="s">
+      <c r="F25" s="11" t="s">
         <v>132</v>
       </c>
-      <c r="G25" s="12" t="s">
+      <c r="G25" s="11" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="26" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B26" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C26" s="12" t="s">
+      <c r="B26" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C26" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="D26" s="12" t="s">
+      <c r="D26" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="E26" s="12"/>
-      <c r="F26" s="12"/>
-      <c r="G26" s="12" t="s">
+      <c r="E26" s="11"/>
+      <c r="F26" s="11"/>
+      <c r="G26" s="11" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="27" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B27" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C27" s="12" t="s">
+      <c r="B27" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C27" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="D27" s="12" t="s">
+      <c r="D27" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="E27" s="12" t="s">
+      <c r="E27" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="F27" s="12"/>
-      <c r="G27" s="12" t="s">
+      <c r="F27" s="11"/>
+      <c r="G27" s="11" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="28" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B28" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C28" s="12" t="s">
+      <c r="B28" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C28" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="D28" s="12" t="s">
+      <c r="D28" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="E28" s="12" t="s">
+      <c r="E28" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="F28" s="12" t="s">
+      <c r="F28" s="11" t="s">
         <v>130</v>
       </c>
-      <c r="G28" s="12" t="s">
+      <c r="G28" s="11" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="29" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B29" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C29" s="12" t="s">
+      <c r="B29" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C29" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="D29" s="12" t="s">
+      <c r="D29" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="E29" s="12"/>
-      <c r="F29" s="12"/>
-      <c r="G29" s="12" t="s">
+      <c r="E29" s="11"/>
+      <c r="F29" s="11"/>
+      <c r="G29" s="11" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="30" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B30" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C30" s="12" t="s">
+      <c r="B30" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C30" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="D30" s="12" t="s">
+      <c r="D30" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="E30" s="12" t="s">
+      <c r="E30" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="G30" s="12" t="s">
+      <c r="G30" s="11" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="31" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B31" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C31" s="12" t="s">
+      <c r="B31" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C31" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="D31" s="12" t="s">
+      <c r="D31" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="E31" s="12" t="s">
+      <c r="E31" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="F31" s="12" t="s">
+      <c r="F31" s="11" t="s">
         <v>129</v>
       </c>
-      <c r="G31" s="12" t="s">
+      <c r="G31" s="11" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B32" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C32" s="12" t="s">
+      <c r="B32" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C32" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="D32" s="12" t="s">
+      <c r="D32" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="E32" s="12"/>
-      <c r="F32" s="12"/>
-      <c r="G32" s="12" t="s">
+      <c r="E32" s="11"/>
+      <c r="F32" s="11"/>
+      <c r="G32" s="11" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="33" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B33" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C33" s="12" t="s">
+      <c r="B33" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C33" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="D33" s="12" t="s">
+      <c r="D33" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="E33" s="12" t="s">
+      <c r="E33" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="F33" s="12"/>
-      <c r="G33" s="12" t="s">
+      <c r="F33" s="11"/>
+      <c r="G33" s="11" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="34" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B34" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C34" s="12" t="s">
+      <c r="B34" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C34" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="D34" s="12" t="s">
+      <c r="D34" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="E34" s="12" t="s">
+      <c r="E34" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="F34" s="12"/>
-      <c r="G34" s="12" t="s">
+      <c r="F34" s="11"/>
+      <c r="G34" s="11" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="35" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B35" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C35" s="12" t="s">
+      <c r="B35" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C35" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="D35" s="12" t="s">
+      <c r="D35" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="E35" s="12" t="s">
+      <c r="E35" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="F35" s="12"/>
-      <c r="G35" s="12" t="s">
+      <c r="F35" s="11"/>
+      <c r="G35" s="11" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="36" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B36" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C36" s="12" t="s">
+      <c r="B36" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C36" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="D36" s="12" t="s">
+      <c r="D36" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="E36" s="12" t="s">
+      <c r="E36" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="F36" s="12"/>
-      <c r="G36" s="12" t="s">
+      <c r="F36" s="11"/>
+      <c r="G36" s="11" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="37" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B37" s="12" t="s">
+      <c r="B37" s="11" t="s">
         <v>177</v>
       </c>
-      <c r="C37" s="12" t="s">
+      <c r="C37" s="11" t="s">
         <v>179</v>
       </c>
-      <c r="D37" s="12" t="s">
+      <c r="D37" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="E37" s="12" t="s">
+      <c r="E37" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="F37" s="13" t="s">
+      <c r="F37" s="12" t="s">
         <v>178</v>
       </c>
-      <c r="G37" s="12" t="s">
+      <c r="G37" s="11" t="s">
         <v>180</v>
       </c>
     </row>
     <row r="38" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B38" s="12" t="s">
+      <c r="B38" s="11" t="s">
         <v>177</v>
       </c>
-      <c r="C38" s="12" t="s">
+      <c r="C38" s="11" t="s">
         <v>198</v>
       </c>
-      <c r="D38" s="12" t="s">
+      <c r="D38" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="E38" s="12" t="s">
+      <c r="E38" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="G38" s="12" t="s">
+      <c r="G38" s="11" t="s">
         <v>229</v>
       </c>
     </row>
     <row r="39" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B39" s="12" t="s">
+      <c r="B39" s="11" t="s">
         <v>177</v>
       </c>
-      <c r="C39" s="12" t="s">
+      <c r="C39" s="11" t="s">
         <v>199</v>
       </c>
-      <c r="D39" s="12" t="s">
+      <c r="D39" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="E39" s="12" t="s">
+      <c r="E39" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="G39" s="12" t="s">
+      <c r="G39" s="11" t="s">
         <v>230</v>
       </c>
     </row>
     <row r="40" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B40" s="12" t="s">
+      <c r="B40" s="11" t="s">
         <v>177</v>
       </c>
-      <c r="C40" s="12" t="s">
+      <c r="C40" s="11" t="s">
         <v>200</v>
       </c>
-      <c r="D40" s="12" t="s">
+      <c r="D40" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="E40" s="12" t="s">
+      <c r="E40" s="11" t="s">
         <v>183</v>
       </c>
-      <c r="F40" s="13" t="s">
+      <c r="F40" s="12" t="s">
         <v>181</v>
       </c>
-      <c r="G40" s="12" t="s">
+      <c r="G40" s="11" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="41" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B41" s="12" t="s">
+      <c r="B41" s="11" t="s">
         <v>177</v>
       </c>
-      <c r="C41" s="12" t="s">
+      <c r="C41" s="11" t="s">
         <v>201</v>
       </c>
-      <c r="D41" s="12" t="s">
+      <c r="D41" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="E41" s="12" t="s">
+      <c r="E41" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="F41" s="13" t="s">
+      <c r="F41" s="12" t="s">
         <v>182</v>
       </c>
-      <c r="G41" s="12" t="s">
+      <c r="G41" s="11" t="s">
         <v>185</v>
       </c>
     </row>
     <row r="42" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B42" s="12" t="s">
+      <c r="B42" s="11" t="s">
         <v>177</v>
       </c>
-      <c r="C42" s="12" t="s">
+      <c r="C42" s="11" t="s">
         <v>227</v>
       </c>
-      <c r="D42" s="12" t="s">
+      <c r="D42" s="11" t="s">
         <v>157</v>
       </c>
-      <c r="E42" s="12"/>
-      <c r="G42" s="12" t="s">
+      <c r="E42" s="11"/>
+      <c r="G42" s="11" t="s">
         <v>228</v>
       </c>
     </row>
     <row r="43" spans="2:7" ht="96" x14ac:dyDescent="0.2">
-      <c r="B43" s="12" t="s">
+      <c r="B43" s="11" t="s">
         <v>177</v>
       </c>
-      <c r="C43" s="12" t="s">
+      <c r="C43" s="11" t="s">
         <v>225</v>
       </c>
-      <c r="D43" s="12" t="s">
+      <c r="D43" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="E43" s="12" t="s">
+      <c r="E43" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="F43" s="14" t="s">
+      <c r="F43" s="13" t="s">
         <v>221</v>
       </c>
-      <c r="G43" s="12" t="s">
+      <c r="G43" s="11" t="s">
         <v>222</v>
       </c>
     </row>
     <row r="44" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B44" s="13" t="s">
-        <v>91</v>
-      </c>
-      <c r="C44" s="13" t="s">
+      <c r="B44" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C44" s="12" t="s">
         <v>243</v>
       </c>
-      <c r="D44" s="13" t="s">
+      <c r="D44" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="E44" s="13" t="s">
+      <c r="E44" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="G44" s="13" t="s">
+      <c r="G44" s="12" t="s">
         <v>244</v>
       </c>
     </row>
     <row r="45" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B45" s="13" t="s">
+      <c r="B45" s="12" t="s">
         <v>248</v>
       </c>
-      <c r="C45" s="13" t="s">
+      <c r="C45" s="12" t="s">
         <v>249</v>
       </c>
-      <c r="D45" s="13" t="s">
+      <c r="D45" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="E45" s="13" t="s">
+      <c r="E45" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="G45" s="13" t="s">
+      <c r="G45" s="12" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="46" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B46" s="13" t="s">
+      <c r="B46" s="12" t="s">
         <v>248</v>
       </c>
-      <c r="C46" s="13" t="s">
+      <c r="C46" s="12" t="s">
         <v>250</v>
       </c>
-      <c r="D46" s="13" t="s">
+      <c r="D46" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="E46" s="13" t="s">
+      <c r="E46" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="G46" s="13" t="s">
+      <c r="G46" s="12" t="s">
         <v>254</v>
       </c>
     </row>
     <row r="47" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B47" s="13" t="s">
+      <c r="B47" s="12" t="s">
         <v>248</v>
       </c>
-      <c r="C47" s="13" t="s">
+      <c r="C47" s="12" t="s">
         <v>251</v>
       </c>
-      <c r="D47" s="13" t="s">
+      <c r="D47" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="E47" s="13" t="s">
+      <c r="E47" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="G47" s="13" t="s">
+      <c r="G47" s="12" t="s">
         <v>255</v>
       </c>
     </row>
     <row r="48" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B48" s="13" t="s">
+      <c r="B48" s="12" t="s">
         <v>248</v>
       </c>
-      <c r="C48" s="13" t="s">
+      <c r="C48" s="12" t="s">
         <v>252</v>
       </c>
-      <c r="D48" s="13" t="s">
+      <c r="D48" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="E48" s="13" t="s">
+      <c r="E48" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="G48" s="13" t="s">
+      <c r="G48" s="12" t="s">
         <v>256</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add lines to capture  mf4 loading errors
</commit_message>
<xml_diff>
--- a/config/kpi_as_long.xlsx
+++ b/config/kpi_as_long.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wangjianhai/02_ADAS/01_repo/01_Tools/01_kpi_extractor/python/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7F9EFD6-A315-1D42-8A61-4EB8487324EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{581AEF62-5882-F24C-9A78-3F4D92CDABC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34200" yWindow="6440" windowWidth="38400" windowHeight="20980" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="700" windowWidth="34200" windowHeight="20520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="params" sheetId="7" r:id="rId1"/>
@@ -917,7 +917,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -950,8 +950,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1799,7 +1797,7 @@
         <v>15</v>
       </c>
       <c r="D2" s="2">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E2" s="2">
         <v>75</v>
@@ -2066,7 +2064,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="2">
-        <v>300</v>
+        <v>450</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>60</v>
@@ -2547,19 +2545,19 @@
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A22" s="14" t="s">
+      <c r="A22" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="B22" s="14" t="s">
+      <c r="B22" s="1" t="s">
         <v>260</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="D22" s="15">
+      <c r="D22" s="2">
         <v>-10</v>
       </c>
-      <c r="E22" s="15">
+      <c r="E22" s="2">
         <v>10</v>
       </c>
       <c r="F22" s="1" t="s">
@@ -2571,7 +2569,7 @@
       <c r="H22" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I22" s="14" t="s">
+      <c r="I22" s="1" t="s">
         <v>256</v>
       </c>
       <c r="J22" s="1" t="s">
@@ -2585,19 +2583,19 @@
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A23" s="14" t="s">
+      <c r="A23" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="B23" s="14" t="s">
+      <c r="B23" s="1" t="s">
         <v>261</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="D23" s="15">
+      <c r="D23" s="2">
         <v>-10</v>
       </c>
-      <c r="E23" s="15">
+      <c r="E23" s="2">
         <v>10</v>
       </c>
       <c r="F23" s="1" t="s">
@@ -2609,7 +2607,7 @@
       <c r="H23" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I23" s="14" t="s">
+      <c r="I23" s="1" t="s">
         <v>257</v>
       </c>
       <c r="J23" s="1" t="s">
@@ -2623,19 +2621,19 @@
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A24" s="14" t="s">
+      <c r="A24" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="B24" s="14" t="s">
+      <c r="B24" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="C24" s="15" t="s">
+      <c r="C24" s="2" t="s">
         <v>250</v>
       </c>
-      <c r="D24" s="15">
+      <c r="D24" s="2">
         <v>-10</v>
       </c>
-      <c r="E24" s="15">
+      <c r="E24" s="2">
         <v>10</v>
       </c>
       <c r="F24" s="1" t="s">
@@ -2647,7 +2645,7 @@
       <c r="H24" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I24" s="14" t="s">
+      <c r="I24" s="1" t="s">
         <v>258</v>
       </c>
       <c r="J24" s="1" t="s">
@@ -2661,19 +2659,19 @@
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A25" s="14" t="s">
+      <c r="A25" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="B25" s="14" t="s">
+      <c r="B25" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="C25" s="15" t="s">
+      <c r="C25" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="D25" s="15">
+      <c r="D25" s="2">
         <v>-10</v>
       </c>
-      <c r="E25" s="15">
+      <c r="E25" s="2">
         <v>10</v>
       </c>
       <c r="F25" s="1" t="s">
@@ -2685,7 +2683,7 @@
       <c r="H25" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I25" s="14" t="s">
+      <c r="I25" s="1" t="s">
         <v>259</v>
       </c>
       <c r="J25" s="1" t="s">

</xml_diff>

<commit_message>
incorporate AS_Long calParam to kpi_as_long.xlsx
</commit_message>
<xml_diff>
--- a/config/kpi_as_long.xlsx
+++ b/config/kpi_as_long.xlsx
@@ -8,17 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wangjianhai/02_ADAS/01_repo/01_Tools/01_kpi_extractor/python/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{347D3AEB-6622-964A-BAC8-064203A1B3F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E73D50A2-EB51-E446-BE50-2DBAA8CF77B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="700" windowWidth="34200" windowHeight="20460" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="420" yWindow="1160" windowWidth="34200" windowHeight="20460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="params" sheetId="7" r:id="rId1"/>
-    <sheet name="graphSpec" sheetId="3" r:id="rId2"/>
-    <sheet name="KPI" sheetId="6" r:id="rId3"/>
-    <sheet name="overallKPI" sheetId="8" r:id="rId4"/>
-    <sheet name="markerShapes" sheetId="5" r:id="rId5"/>
-    <sheet name="lineColors" sheetId="4" r:id="rId6"/>
+    <sheet name="calParam" sheetId="9" r:id="rId2"/>
+    <sheet name="graphSpec" sheetId="3" r:id="rId3"/>
+    <sheet name="KPI" sheetId="6" r:id="rId4"/>
+    <sheet name="overallKPI" sheetId="8" r:id="rId5"/>
+    <sheet name="markerShapes" sheetId="5" r:id="rId6"/>
+    <sheet name="lineColors" sheetId="4" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="636" uniqueCount="289">
   <si>
     <t>Reference</t>
   </si>
@@ -872,6 +873,45 @@
   </si>
   <si>
     <t>CPM_ACT</t>
+  </si>
+  <si>
+    <t>Yaw_rate</t>
+  </si>
+  <si>
+    <t>egoSpd</t>
+  </si>
+  <si>
+    <t>Base</t>
+  </si>
+  <si>
+    <t>Cal1</t>
+  </si>
+  <si>
+    <t>Cal2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lateral_acceleration </t>
+  </si>
+  <si>
+    <t>base</t>
+  </si>
+  <si>
+    <t>cal1</t>
+  </si>
+  <si>
+    <t>cal2</t>
+  </si>
+  <si>
+    <t>Steering_wheel</t>
+  </si>
+  <si>
+    <t>PedalPosPro_Override</t>
+  </si>
+  <si>
+    <t>PedalPosPro_th</t>
+  </si>
+  <si>
+    <t>Throttle</t>
   </si>
 </sst>
 </file>
@@ -916,12 +956,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF6F900"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -951,7 +997,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -984,12 +1030,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFF6F900"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1766,6 +1823,945 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49B0BB4F-1B00-0B46-A628-68556F5EA1D3}">
+  <dimension ref="B2:AF36"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="8.83203125" customWidth="1"/>
+    <col min="3" max="8" width="5.83203125" customWidth="1"/>
+    <col min="9" max="9" width="2.83203125" customWidth="1"/>
+    <col min="10" max="10" width="8.83203125" customWidth="1"/>
+    <col min="11" max="22" width="5.83203125" customWidth="1"/>
+    <col min="25" max="31" width="6.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:29" x14ac:dyDescent="0.2">
+      <c r="B2" t="s">
+        <v>276</v>
+      </c>
+      <c r="J2" t="s">
+        <v>285</v>
+      </c>
+      <c r="X2" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="3" spans="2:29" x14ac:dyDescent="0.2">
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="J3" t="s">
+        <v>9</v>
+      </c>
+      <c r="X3" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="4" spans="2:29" x14ac:dyDescent="0.2">
+      <c r="B4" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="C4" s="1">
+        <v>5</v>
+      </c>
+      <c r="D4" s="1">
+        <v>15</v>
+      </c>
+      <c r="E4" s="1">
+        <v>40</v>
+      </c>
+      <c r="F4" s="1">
+        <v>65</v>
+      </c>
+      <c r="G4" s="1">
+        <v>80</v>
+      </c>
+      <c r="H4" s="1">
+        <v>100</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="K4" s="1">
+        <v>0</v>
+      </c>
+      <c r="L4" s="1">
+        <v>10</v>
+      </c>
+      <c r="M4" s="1">
+        <v>25</v>
+      </c>
+      <c r="N4" s="1">
+        <v>30</v>
+      </c>
+      <c r="O4" s="1">
+        <v>35</v>
+      </c>
+      <c r="P4" s="1">
+        <v>40</v>
+      </c>
+      <c r="Q4" s="1">
+        <v>45</v>
+      </c>
+      <c r="R4" s="1">
+        <v>50</v>
+      </c>
+      <c r="S4" s="1">
+        <v>55</v>
+      </c>
+      <c r="T4" s="1">
+        <v>60</v>
+      </c>
+      <c r="U4" s="1">
+        <v>130</v>
+      </c>
+      <c r="V4" s="1">
+        <v>250</v>
+      </c>
+      <c r="X4" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="Y4" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z4" s="1">
+        <v>10</v>
+      </c>
+      <c r="AA4" s="1">
+        <v>20</v>
+      </c>
+      <c r="AB4" s="1">
+        <v>30</v>
+      </c>
+      <c r="AC4" s="1">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="5" spans="2:29" x14ac:dyDescent="0.2">
+      <c r="B5" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="C5" s="1">
+        <v>42</v>
+      </c>
+      <c r="D5" s="1">
+        <v>42</v>
+      </c>
+      <c r="E5" s="1">
+        <v>21</v>
+      </c>
+      <c r="F5" s="1">
+        <v>14</v>
+      </c>
+      <c r="G5" s="1">
+        <v>11</v>
+      </c>
+      <c r="H5" s="1">
+        <v>11</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="K5" s="1">
+        <v>360</v>
+      </c>
+      <c r="L5" s="1">
+        <v>270</v>
+      </c>
+      <c r="M5" s="1">
+        <v>222</v>
+      </c>
+      <c r="N5" s="1">
+        <v>175</v>
+      </c>
+      <c r="O5" s="1">
+        <v>127</v>
+      </c>
+      <c r="P5" s="1">
+        <v>80</v>
+      </c>
+      <c r="Q5" s="1">
+        <v>75</v>
+      </c>
+      <c r="R5" s="1">
+        <v>70</v>
+      </c>
+      <c r="S5" s="1">
+        <v>65</v>
+      </c>
+      <c r="T5" s="1">
+        <v>60</v>
+      </c>
+      <c r="U5" s="1">
+        <v>60</v>
+      </c>
+      <c r="V5" s="1">
+        <v>60</v>
+      </c>
+      <c r="X5" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="Y5" s="17">
+        <v>50</v>
+      </c>
+      <c r="Z5" s="17">
+        <v>50</v>
+      </c>
+      <c r="AA5" s="17">
+        <v>50</v>
+      </c>
+      <c r="AB5" s="17">
+        <v>50</v>
+      </c>
+      <c r="AC5" s="17">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="2:29" x14ac:dyDescent="0.2">
+      <c r="B6" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="C6" s="1">
+        <v>5</v>
+      </c>
+      <c r="D6" s="1">
+        <v>20</v>
+      </c>
+      <c r="E6" s="1">
+        <v>40</v>
+      </c>
+      <c r="F6" s="1">
+        <v>55</v>
+      </c>
+      <c r="G6" s="1">
+        <v>65</v>
+      </c>
+      <c r="H6" s="1">
+        <v>80</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="K6" s="1">
+        <v>0</v>
+      </c>
+      <c r="L6" s="1">
+        <v>10</v>
+      </c>
+      <c r="M6" s="1">
+        <v>15</v>
+      </c>
+      <c r="N6" s="1">
+        <v>20</v>
+      </c>
+      <c r="O6" s="1">
+        <v>30</v>
+      </c>
+      <c r="P6" s="1">
+        <v>35</v>
+      </c>
+      <c r="Q6" s="1">
+        <v>40</v>
+      </c>
+      <c r="R6" s="1">
+        <v>45</v>
+      </c>
+      <c r="S6" s="1">
+        <v>50</v>
+      </c>
+      <c r="T6" s="1">
+        <v>55</v>
+      </c>
+      <c r="U6" s="1">
+        <v>70</v>
+      </c>
+      <c r="V6" s="1">
+        <v>80</v>
+      </c>
+      <c r="X6" s="14" t="s">
+        <v>277</v>
+      </c>
+      <c r="Y6" s="14">
+        <v>0</v>
+      </c>
+      <c r="Z6" s="14">
+        <v>10</v>
+      </c>
+      <c r="AA6" s="14">
+        <v>20</v>
+      </c>
+      <c r="AB6" s="14">
+        <v>65</v>
+      </c>
+      <c r="AC6" s="14">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="2:29" x14ac:dyDescent="0.2">
+      <c r="B7" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="C7" s="1">
+        <v>12</v>
+      </c>
+      <c r="D7" s="1">
+        <v>16</v>
+      </c>
+      <c r="E7" s="1">
+        <v>17</v>
+      </c>
+      <c r="F7" s="1">
+        <v>18</v>
+      </c>
+      <c r="G7" s="1">
+        <v>18.5</v>
+      </c>
+      <c r="H7" s="1">
+        <v>19</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="K7" s="1">
+        <v>220</v>
+      </c>
+      <c r="L7" s="1">
+        <v>210</v>
+      </c>
+      <c r="M7" s="1">
+        <v>170</v>
+      </c>
+      <c r="N7" s="1">
+        <v>130</v>
+      </c>
+      <c r="O7" s="1">
+        <v>95</v>
+      </c>
+      <c r="P7" s="1">
+        <v>80</v>
+      </c>
+      <c r="Q7" s="1">
+        <v>70</v>
+      </c>
+      <c r="R7" s="1">
+        <v>65</v>
+      </c>
+      <c r="S7" s="1">
+        <v>63</v>
+      </c>
+      <c r="T7" s="1">
+        <v>60</v>
+      </c>
+      <c r="U7" s="1">
+        <v>58</v>
+      </c>
+      <c r="V7" s="1">
+        <v>55</v>
+      </c>
+      <c r="X7" s="14" t="s">
+        <v>283</v>
+      </c>
+      <c r="Y7" s="19">
+        <v>60</v>
+      </c>
+      <c r="Z7" s="19">
+        <v>65</v>
+      </c>
+      <c r="AA7" s="19">
+        <v>70</v>
+      </c>
+      <c r="AB7" s="19">
+        <v>70</v>
+      </c>
+      <c r="AC7" s="19">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="8" spans="2:29" x14ac:dyDescent="0.2">
+      <c r="B8" s="14" t="s">
+        <v>277</v>
+      </c>
+      <c r="C8" s="14">
+        <v>5</v>
+      </c>
+      <c r="D8" s="14">
+        <v>22</v>
+      </c>
+      <c r="E8" s="14">
+        <v>40</v>
+      </c>
+      <c r="F8" s="14">
+        <v>55</v>
+      </c>
+      <c r="G8" s="14">
+        <v>65</v>
+      </c>
+      <c r="H8" s="14">
+        <v>80</v>
+      </c>
+      <c r="J8" s="14" t="s">
+        <v>277</v>
+      </c>
+      <c r="K8" s="14">
+        <v>5</v>
+      </c>
+      <c r="L8" s="14">
+        <v>10</v>
+      </c>
+      <c r="M8" s="14">
+        <v>15</v>
+      </c>
+      <c r="N8" s="14">
+        <v>20</v>
+      </c>
+      <c r="O8" s="14">
+        <v>28</v>
+      </c>
+      <c r="P8" s="14">
+        <v>35</v>
+      </c>
+      <c r="Q8" s="14">
+        <v>40</v>
+      </c>
+      <c r="R8" s="14">
+        <v>45</v>
+      </c>
+      <c r="S8" s="14">
+        <v>50</v>
+      </c>
+      <c r="T8" s="14">
+        <v>55</v>
+      </c>
+      <c r="U8" s="14">
+        <v>70</v>
+      </c>
+      <c r="V8" s="14">
+        <v>80</v>
+      </c>
+      <c r="Y8" s="16"/>
+      <c r="Z8" s="16"/>
+      <c r="AA8" s="16"/>
+      <c r="AB8" s="16"/>
+      <c r="AC8" s="16"/>
+    </row>
+    <row r="9" spans="2:29" x14ac:dyDescent="0.2">
+      <c r="B9" s="14" t="s">
+        <v>280</v>
+      </c>
+      <c r="C9" s="14">
+        <v>40</v>
+      </c>
+      <c r="D9" s="14">
+        <v>40</v>
+      </c>
+      <c r="E9" s="14">
+        <v>20</v>
+      </c>
+      <c r="F9" s="14">
+        <v>19</v>
+      </c>
+      <c r="G9" s="14">
+        <v>18</v>
+      </c>
+      <c r="H9" s="14">
+        <v>18</v>
+      </c>
+      <c r="J9" s="14" t="s">
+        <v>284</v>
+      </c>
+      <c r="K9" s="14">
+        <v>430</v>
+      </c>
+      <c r="L9" s="14">
+        <v>430</v>
+      </c>
+      <c r="M9" s="14">
+        <v>400</v>
+      </c>
+      <c r="N9" s="14">
+        <v>350</v>
+      </c>
+      <c r="O9" s="14">
+        <v>200</v>
+      </c>
+      <c r="P9" s="14">
+        <v>100</v>
+      </c>
+      <c r="Q9" s="14">
+        <v>70</v>
+      </c>
+      <c r="R9" s="14">
+        <v>65</v>
+      </c>
+      <c r="S9" s="14">
+        <v>63</v>
+      </c>
+      <c r="T9" s="14">
+        <v>60</v>
+      </c>
+      <c r="U9" s="14">
+        <v>58</v>
+      </c>
+      <c r="V9" s="14">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="10" spans="2:29" x14ac:dyDescent="0.2">
+      <c r="Y10" s="16"/>
+      <c r="Z10" s="16"/>
+      <c r="AA10" s="16"/>
+      <c r="AB10" s="16"/>
+      <c r="AC10" s="16"/>
+    </row>
+    <row r="11" spans="2:29" x14ac:dyDescent="0.2">
+      <c r="Y11" s="16"/>
+      <c r="Z11" s="16"/>
+      <c r="AA11" s="16"/>
+      <c r="AB11" s="16"/>
+      <c r="AC11" s="16"/>
+    </row>
+    <row r="12" spans="2:29" x14ac:dyDescent="0.2">
+      <c r="Y12" s="16"/>
+      <c r="Z12" s="16"/>
+      <c r="AA12" s="16"/>
+      <c r="AB12" s="16"/>
+      <c r="AC12" s="16"/>
+    </row>
+    <row r="13" spans="2:29" x14ac:dyDescent="0.2">
+      <c r="B13" t="s">
+        <v>281</v>
+      </c>
+      <c r="Y13" s="16"/>
+      <c r="Z13" s="16"/>
+      <c r="AA13" s="16"/>
+      <c r="AB13" s="16"/>
+      <c r="AC13" s="16"/>
+    </row>
+    <row r="14" spans="2:29" x14ac:dyDescent="0.2">
+      <c r="B14" t="s">
+        <v>12</v>
+      </c>
+      <c r="J14" t="s">
+        <v>10</v>
+      </c>
+      <c r="X14" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="2:29" x14ac:dyDescent="0.2">
+      <c r="B15" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="C15" s="1">
+        <v>5</v>
+      </c>
+      <c r="D15" s="1">
+        <v>15</v>
+      </c>
+      <c r="E15" s="1">
+        <v>40</v>
+      </c>
+      <c r="F15" s="1">
+        <v>65</v>
+      </c>
+      <c r="G15" s="1">
+        <v>80</v>
+      </c>
+      <c r="H15" s="1">
+        <v>100</v>
+      </c>
+      <c r="J15" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="K15" s="1">
+        <v>5</v>
+      </c>
+      <c r="L15" s="1">
+        <v>15</v>
+      </c>
+      <c r="M15" s="1">
+        <v>40</v>
+      </c>
+      <c r="N15" s="1">
+        <v>65</v>
+      </c>
+      <c r="O15" s="1">
+        <v>80</v>
+      </c>
+      <c r="P15" s="1">
+        <v>100</v>
+      </c>
+      <c r="Q15" s="1"/>
+      <c r="R15" s="1"/>
+      <c r="S15" s="1"/>
+      <c r="T15" s="1"/>
+      <c r="U15" s="1"/>
+      <c r="V15" s="1"/>
+      <c r="X15" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="Y15" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z15" s="1">
+        <v>10</v>
+      </c>
+      <c r="AA15" s="1">
+        <v>20</v>
+      </c>
+      <c r="AB15" s="1">
+        <v>30</v>
+      </c>
+      <c r="AC15" s="1">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="16" spans="2:29" x14ac:dyDescent="0.2">
+      <c r="B16" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="C16" s="1">
+        <v>4</v>
+      </c>
+      <c r="D16" s="1">
+        <v>4</v>
+      </c>
+      <c r="E16" s="1">
+        <v>4</v>
+      </c>
+      <c r="F16" s="1">
+        <v>4</v>
+      </c>
+      <c r="G16" s="1">
+        <v>4</v>
+      </c>
+      <c r="H16" s="1">
+        <v>4</v>
+      </c>
+      <c r="J16" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="K16" s="1">
+        <v>100</v>
+      </c>
+      <c r="L16" s="1">
+        <v>100</v>
+      </c>
+      <c r="M16" s="1">
+        <v>100</v>
+      </c>
+      <c r="N16" s="1">
+        <v>100</v>
+      </c>
+      <c r="O16" s="1">
+        <v>100</v>
+      </c>
+      <c r="P16" s="1">
+        <v>100</v>
+      </c>
+      <c r="Q16" s="1"/>
+      <c r="R16" s="1"/>
+      <c r="S16" s="1"/>
+      <c r="T16" s="1"/>
+      <c r="U16" s="1"/>
+      <c r="V16" s="1"/>
+      <c r="X16" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="Y16" s="1">
+        <v>20</v>
+      </c>
+      <c r="Z16" s="1">
+        <v>20</v>
+      </c>
+      <c r="AA16" s="1">
+        <v>20</v>
+      </c>
+      <c r="AB16" s="1">
+        <v>30</v>
+      </c>
+      <c r="AC16" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17" spans="2:31" x14ac:dyDescent="0.2">
+      <c r="B17" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="C17" s="1">
+        <v>5</v>
+      </c>
+      <c r="D17" s="1">
+        <v>15</v>
+      </c>
+      <c r="E17" s="1">
+        <v>30</v>
+      </c>
+      <c r="F17" s="1">
+        <v>45</v>
+      </c>
+      <c r="G17" s="1">
+        <v>65</v>
+      </c>
+      <c r="H17" s="1">
+        <v>80</v>
+      </c>
+      <c r="J17" s="14" t="s">
+        <v>277</v>
+      </c>
+      <c r="K17" s="14">
+        <v>0</v>
+      </c>
+      <c r="L17" s="14">
+        <v>10</v>
+      </c>
+      <c r="M17" s="14">
+        <v>15</v>
+      </c>
+      <c r="N17" s="14">
+        <v>20</v>
+      </c>
+      <c r="O17" s="14">
+        <v>25</v>
+      </c>
+      <c r="P17" s="14">
+        <v>30</v>
+      </c>
+      <c r="Q17" s="14">
+        <v>35</v>
+      </c>
+      <c r="R17" s="14">
+        <v>40</v>
+      </c>
+      <c r="S17" s="14">
+        <v>50</v>
+      </c>
+      <c r="T17" s="14">
+        <v>55</v>
+      </c>
+      <c r="U17" s="14">
+        <v>70</v>
+      </c>
+      <c r="V17" s="14">
+        <v>80</v>
+      </c>
+      <c r="X17" s="14" t="s">
+        <v>277</v>
+      </c>
+      <c r="Y17" s="14">
+        <v>0</v>
+      </c>
+      <c r="Z17" s="14">
+        <v>10</v>
+      </c>
+      <c r="AA17" s="14">
+        <v>20</v>
+      </c>
+      <c r="AB17" s="14">
+        <v>65</v>
+      </c>
+      <c r="AC17" s="14">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18" spans="2:31" x14ac:dyDescent="0.2">
+      <c r="B18" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="C18" s="1">
+        <v>1.7</v>
+      </c>
+      <c r="D18" s="1">
+        <v>2.5</v>
+      </c>
+      <c r="E18" s="1">
+        <v>3.3</v>
+      </c>
+      <c r="F18" s="1">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="G18" s="1">
+        <v>4.8</v>
+      </c>
+      <c r="H18" s="1">
+        <v>5.2</v>
+      </c>
+      <c r="J18" s="14" t="s">
+        <v>283</v>
+      </c>
+      <c r="K18" s="14">
+        <v>580</v>
+      </c>
+      <c r="L18" s="14">
+        <v>570</v>
+      </c>
+      <c r="M18" s="14">
+        <v>430</v>
+      </c>
+      <c r="N18" s="14">
+        <v>390</v>
+      </c>
+      <c r="O18" s="14">
+        <v>350</v>
+      </c>
+      <c r="P18" s="14">
+        <v>330</v>
+      </c>
+      <c r="Q18" s="14">
+        <v>310</v>
+      </c>
+      <c r="R18" s="14">
+        <v>295</v>
+      </c>
+      <c r="S18" s="14">
+        <v>260</v>
+      </c>
+      <c r="T18" s="14">
+        <v>250</v>
+      </c>
+      <c r="U18" s="14">
+        <v>245</v>
+      </c>
+      <c r="V18" s="14">
+        <v>240</v>
+      </c>
+      <c r="X18" s="14" t="s">
+        <v>283</v>
+      </c>
+      <c r="Y18" s="14">
+        <v>55</v>
+      </c>
+      <c r="Z18" s="14">
+        <v>60</v>
+      </c>
+      <c r="AA18" s="14">
+        <v>65</v>
+      </c>
+      <c r="AB18" s="14">
+        <v>65</v>
+      </c>
+      <c r="AC18" s="14">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="19" spans="2:31" x14ac:dyDescent="0.2">
+      <c r="B19" s="14" t="s">
+        <v>277</v>
+      </c>
+      <c r="C19" s="14">
+        <v>5</v>
+      </c>
+      <c r="D19" s="14">
+        <v>15</v>
+      </c>
+      <c r="E19" s="14">
+        <v>25</v>
+      </c>
+      <c r="F19" s="14">
+        <v>45</v>
+      </c>
+      <c r="G19" s="14">
+        <v>65</v>
+      </c>
+      <c r="H19" s="14">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="20" spans="2:31" x14ac:dyDescent="0.2">
+      <c r="B20" s="14" t="s">
+        <v>280</v>
+      </c>
+      <c r="C20" s="14">
+        <v>2.8</v>
+      </c>
+      <c r="D20" s="14">
+        <v>4.3</v>
+      </c>
+      <c r="E20" s="14">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="F20" s="14">
+        <v>5.4</v>
+      </c>
+      <c r="G20" s="14">
+        <v>5.5</v>
+      </c>
+      <c r="H20" s="14">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="24" spans="2:31" x14ac:dyDescent="0.2">
+      <c r="X24" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="25" spans="2:31" x14ac:dyDescent="0.2">
+      <c r="X25" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="Y25" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z25" s="1">
+        <v>20</v>
+      </c>
+      <c r="AA25" s="1">
+        <v>40</v>
+      </c>
+      <c r="AB25" s="1">
+        <v>60</v>
+      </c>
+      <c r="AC25" s="1">
+        <v>80</v>
+      </c>
+      <c r="AD25" s="1">
+        <v>130</v>
+      </c>
+      <c r="AE25" s="1">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="26" spans="2:31" x14ac:dyDescent="0.2">
+      <c r="X26" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="Y26" s="18">
+        <v>85</v>
+      </c>
+      <c r="Z26" s="18">
+        <v>85</v>
+      </c>
+      <c r="AA26" s="18">
+        <v>85</v>
+      </c>
+      <c r="AB26" s="18">
+        <v>85</v>
+      </c>
+      <c r="AC26" s="18">
+        <v>85</v>
+      </c>
+      <c r="AD26" s="18">
+        <v>85</v>
+      </c>
+      <c r="AE26" s="18">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="36" spans="26:32" x14ac:dyDescent="0.2">
+      <c r="Z36" s="15"/>
+      <c r="AA36" s="15"/>
+      <c r="AB36" s="15"/>
+      <c r="AC36" s="15"/>
+      <c r="AD36" s="15"/>
+      <c r="AE36" s="15"/>
+      <c r="AF36" s="15"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24310F59-1486-4F41-B3B7-AB25CE8F592D}">
   <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -2749,7 +3745,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CE39B99-0AFB-8547-83BF-D855CC6E3BB3}">
   <dimension ref="B1:G48"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -3622,7 +4618,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5705F2F5-A4FE-CE49-A935-9D51D28B5CFA}">
   <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -3763,7 +4759,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA1821CB-8E60-1A45-8122-C329B6E1FCF3}">
   <dimension ref="B1:B9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -3818,7 +4814,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F1943DE-263B-CE4F-869C-DE791D333F1F}">
   <dimension ref="B2:F9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>

</xml_diff>